<commit_message>
feat(auth): add JWT token to Authorization header across all API calls
- Add Authorization header with JWT token to all fetch requests in component API calls
- Update AdminDashboard activity logs endpoint to include Authorization header
- Update BulkUploadModal createBulkTests endpoint to pass JWT in header
- Update CandidateApplyModal to include Authorization header in all API requests (getJD, saveJD, saveThreshold, list, generateReport, checkTestStatus, checkResult)
- Update CandidateSpecificTestModal to include Authorization header in template questions and keyword extraction endpoints
- Update remaining components to consistently pass JWT token via Authorization header instead of request body
- Update activity logger and template history logger utilities to support Authorization header pattern
- Update API inventory documentation with header requirements
- Standardizes authentication across all API integrations following security best practices
</commit_message>
<xml_diff>
--- a/HRRobots_API_Inventory.xlsx
+++ b/HRRobots_API_Inventory.xlsx
@@ -149,7 +149,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -171,11 +171,17 @@
         <color rgb="00AAAAAA"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -303,6 +309,21 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -669,7 +690,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J53"/>
+  <dimension ref="A1:J60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3336,6 +3357,356 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" s="44" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="45" t="inlineStr">
+        <is>
+          <t>Admin / Maintenance</t>
+        </is>
+      </c>
+      <c r="C54" s="44" t="inlineStr">
+        <is>
+          <t>Delete ALL Test Transactions</t>
+        </is>
+      </c>
+      <c r="D54" s="44" t="inlineStr">
+        <is>
+          <t>https://yrtfujcubk4z7pnpynlrfd7isa0farpg.lambda-url.us-east-1.on.aws/</t>
+        </is>
+      </c>
+      <c r="E54" s="46" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="F54" s="44" t="inlineStr">
+        <is>
+          <t>Lambda URL</t>
+        </is>
+      </c>
+      <c r="G54" s="47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H54" s="48" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I54" s="44" t="inlineStr">
+        <is>
+          <t>CRITICAL: Permanently deletes ALL test transaction records and ALL associated candidate photos from S3. Irreversible.</t>
+        </is>
+      </c>
+      <c r="J54" s="44" t="inlineStr">
+        <is>
+          <t>AdminCleanup.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="44" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="45" t="inlineStr">
+        <is>
+          <t>Admin / Maintenance</t>
+        </is>
+      </c>
+      <c r="C55" s="44" t="inlineStr">
+        <is>
+          <t>Delete All MCQ Answers</t>
+        </is>
+      </c>
+      <c r="D55" s="44" t="inlineStr">
+        <is>
+          <t>https://5v3zsgkuuipdy7622htjjixofe0aqtag.lambda-url.us-east-1.on.aws/</t>
+        </is>
+      </c>
+      <c r="E55" s="46" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="F55" s="44" t="inlineStr">
+        <is>
+          <t>Lambda URL</t>
+        </is>
+      </c>
+      <c r="G55" s="47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H55" s="48" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I55" s="44" t="inlineStr">
+        <is>
+          <t>Removes all records from the MCQAnswers table. Destructive and irreversible.</t>
+        </is>
+      </c>
+      <c r="J55" s="44" t="inlineStr">
+        <is>
+          <t>AdminCleanup.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="44" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="45" t="inlineStr">
+        <is>
+          <t>Admin / Maintenance</t>
+        </is>
+      </c>
+      <c r="C56" s="44" t="inlineStr">
+        <is>
+          <t>Clean Orphaned Questions</t>
+        </is>
+      </c>
+      <c r="D56" s="44" t="inlineStr">
+        <is>
+          <t>https://llqoitnux26tdtzpfhnktwha4i0jusof.lambda-url.us-east-1.on.aws/</t>
+        </is>
+      </c>
+      <c r="E56" s="46" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="F56" s="44" t="inlineStr">
+        <is>
+          <t>Lambda URL</t>
+        </is>
+      </c>
+      <c r="G56" s="47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H56" s="48" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I56" s="44" t="inlineStr">
+        <is>
+          <t>Deletes MCQ questions referencing non-existent templates and answers linked to non-existent questions.</t>
+        </is>
+      </c>
+      <c r="J56" s="44" t="inlineStr">
+        <is>
+          <t>AdminCleanup.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="44" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="45" t="inlineStr">
+        <is>
+          <t>Admin / Maintenance</t>
+        </is>
+      </c>
+      <c r="C57" s="44" t="inlineStr">
+        <is>
+          <t>Delete ALL Orphaned Questions</t>
+        </is>
+      </c>
+      <c r="D57" s="44" t="inlineStr">
+        <is>
+          <t>https://mw5cnwjco4rcvjznxbkgexyuny0dkinf.lambda-url.us-east-1.on.aws/</t>
+        </is>
+      </c>
+      <c r="E57" s="46" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="F57" s="44" t="inlineStr">
+        <is>
+          <t>Lambda URL</t>
+        </is>
+      </c>
+      <c r="G57" s="47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H57" s="48" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I57" s="44" t="inlineStr">
+        <is>
+          <t>Comprehensive cleanup: removes all orphaned questions and answers with invalid template/question references.</t>
+        </is>
+      </c>
+      <c r="J57" s="44" t="inlineStr">
+        <is>
+          <t>AdminCleanup.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="44" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="45" t="inlineStr">
+        <is>
+          <t>Admin / Maintenance</t>
+        </is>
+      </c>
+      <c r="C58" s="44" t="inlineStr">
+        <is>
+          <t>Clean Orphaned Test Transactions</t>
+        </is>
+      </c>
+      <c r="D58" s="44" t="inlineStr">
+        <is>
+          <t>https://rnsj7itnilojoqbrbiegjaydbu0yiyeu.lambda-url.us-east-1.on.aws/</t>
+        </is>
+      </c>
+      <c r="E58" s="46" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="F58" s="44" t="inlineStr">
+        <is>
+          <t>Lambda URL</t>
+        </is>
+      </c>
+      <c r="G58" s="47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H58" s="48" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I58" s="44" t="inlineStr">
+        <is>
+          <t>Removes test transactions referencing templates that no longer exist.</t>
+        </is>
+      </c>
+      <c r="J58" s="44" t="inlineStr">
+        <is>
+          <t>AdminCleanup.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="44" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="45" t="inlineStr">
+        <is>
+          <t>Admin / Maintenance</t>
+        </is>
+      </c>
+      <c r="C59" s="44" t="inlineStr">
+        <is>
+          <t>Clean Orphaned Photo Records</t>
+        </is>
+      </c>
+      <c r="D59" s="44" t="inlineStr">
+        <is>
+          <t>https://aavtelreorhxcrf25475eva6mm0eaudo.lambda-url.us-east-1.on.aws/</t>
+        </is>
+      </c>
+      <c r="E59" s="46" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="F59" s="44" t="inlineStr">
+        <is>
+          <t>Lambda URL</t>
+        </is>
+      </c>
+      <c r="G59" s="47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H59" s="48" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I59" s="44" t="inlineStr">
+        <is>
+          <t>Deletes candidatePhoto records where the associated S3 image file no longer exists (s3://hrrfiles).</t>
+        </is>
+      </c>
+      <c r="J59" s="44" t="inlineStr">
+        <is>
+          <t>AdminCleanup.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="44" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="45" t="inlineStr">
+        <is>
+          <t>Admin / Maintenance</t>
+        </is>
+      </c>
+      <c r="C60" s="44" t="inlineStr">
+        <is>
+          <t>Test Auth Endpoint (debug)</t>
+        </is>
+      </c>
+      <c r="D60" s="44" t="inlineStr">
+        <is>
+          <t>https://wssmlq04ef.execute-api.us-east-1.amazonaws.com/test/test</t>
+        </is>
+      </c>
+      <c r="E60" s="46" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="F60" s="44" t="inlineStr">
+        <is>
+          <t>wssmlq04ef</t>
+        </is>
+      </c>
+      <c r="G60" s="47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H60" s="48" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I60" s="44" t="inlineStr">
+        <is>
+          <t>Dev/debug test endpoint. Not used in production flows.</t>
+        </is>
+      </c>
+      <c r="J60" s="44" t="inlineStr">
+        <is>
+          <t>testAuth.js</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3347,7 +3718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -3361,6 +3732,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -3384,132 +3756,143 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Admin / Maintenance</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>Answers &amp; Scoring</t>
         </is>
       </c>
-      <c r="B5" s="14" t="n">
+      <c r="B6" s="14" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Authentication</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n">
+      <c r="B7" s="2" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="33" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="33" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="B7" s="32" t="n">
+      <c r="B8" s="32" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="36" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="36" t="inlineStr">
         <is>
           <t>Feedback</t>
         </is>
       </c>
-      <c r="B8" s="35" t="n">
+      <c r="B9" s="35" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="27" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="27" t="inlineStr">
         <is>
           <t>Logging</t>
         </is>
       </c>
-      <c r="B9" s="26" t="n">
+      <c r="B10" s="26" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="24" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="24" t="inlineStr">
         <is>
           <t>Proctor</t>
         </is>
       </c>
-      <c r="B10" s="23" t="n">
+      <c r="B11" s="23" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>Questions</t>
         </is>
       </c>
-      <c r="B11" s="11" t="n">
+      <c r="B12" s="11" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="30" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="30" t="inlineStr">
         <is>
           <t>Resume / JD</t>
         </is>
       </c>
-      <c r="B12" s="29" t="n">
+      <c r="B13" s="29" t="n">
         <v>6</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="18" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>Templates</t>
         </is>
       </c>
-      <c r="B13" s="17" t="n">
+      <c r="B14" s="17" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>Test Management</t>
         </is>
       </c>
-      <c r="B14" s="8" t="n">
+      <c r="B15" s="8" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="39" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="39" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B15" s="39" t="n">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="40" t="inlineStr">
+      <c r="B16" s="39" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" s="40" t="inlineStr">
         <is>
           <t>In-Session APIs</t>
         </is>
       </c>
-      <c r="B17" s="41" t="n">
+      <c r="B18" s="41" t="n">
         <v>13</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="42" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="42" t="inlineStr">
         <is>
           <t>Out-Session APIs</t>
         </is>
       </c>
-      <c r="B18" s="43" t="n">
+      <c r="B19" s="43" t="n">
         <v>43</v>
       </c>
     </row>

</xml_diff>